<commit_message>
Corregir tres bugs visuales de RESERVAS.
- Botón ESTADO DE CUENTA: descubre el PDF oficial del comunicado más
  reciente de Banxico y valida que responda HTTP 200; si falla, usa la
  página estable del estado de cuenta semanal.
- Color del saldo en la tarjeta oscura: elimina el estilo inline
  `saldoColor` y deja que la regla `.mini.dark .num { color: #fff; }`
  haga herencia; añade `color: inherit` a `.mini .num`.
- Texto duplicado "Semana al": normaliza periodo a "Semana al 28 Ago 26",
  lo muestra en mayúsculas en la tarjeta Panorama y en ficha sin repetir.
- Actualiza tests/test_reservas.py con cobertura de URL 200, herencia de
  color y ausencia de duplicado.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/downloads/indicadores/RESERVAS/RESERVAS_datos.xlsx
+++ b/downloads/indicadores/RESERVAS/RESERVAS_datos.xlsx
@@ -510,7 +510,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>URL del boletín / serie: https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/ · Fecha de publicación: —</t>
+          <t>URL del boletín / serie: https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf · Fecha de publicación: —</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J6" s="8" t="inlineStr">
@@ -627,7 +627,7 @@
       </c>
       <c r="I7" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J7" s="12" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J10" s="8" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J11" s="12" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J12" s="8" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J13" s="12" t="inlineStr">
@@ -879,7 +879,7 @@
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J14" s="8" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J16" s="8" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J17" s="12" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J18" s="8" t="inlineStr">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="I19" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J19" s="12" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J20" s="8" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="I21" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J21" s="12" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J22" s="8" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="I23" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J23" s="12" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J24" s="8" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="I25" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J25" s="12" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="I26" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J26" s="8" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="I27" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J27" s="12" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J28" s="8" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="I29" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J29" s="12" t="inlineStr">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J30" s="8" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="I31" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J31" s="12" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J32" s="8" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="I33" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J33" s="12" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J34" s="8" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="I35" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J35" s="12" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J36" s="8" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="I37" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J37" s="12" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="I38" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J38" s="8" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="I39" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J39" s="12" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="I40" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J40" s="8" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="I41" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J41" s="12" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="I42" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J42" s="8" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="I43" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J43" s="12" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="I44" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J44" s="8" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="I45" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J45" s="12" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="I46" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J46" s="8" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="I47" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J47" s="12" t="inlineStr">
@@ -2103,7 +2103,7 @@
       </c>
       <c r="I48" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J48" s="8" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="I49" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J49" s="12" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="I50" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J50" s="8" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="I51" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J51" s="12" t="inlineStr">
@@ -2247,7 +2247,7 @@
       </c>
       <c r="I52" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J52" s="8" t="inlineStr">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="I53" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J53" s="12" t="inlineStr">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="I54" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J54" s="8" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="I55" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J55" s="12" t="inlineStr">
@@ -2391,7 +2391,7 @@
       </c>
       <c r="I56" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J56" s="8" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="I57" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J57" s="12" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="I58" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J58" s="8" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="I59" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J59" s="12" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="I60" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J60" s="8" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="I61" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J61" s="12" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="I62" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J62" s="8" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="I63" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J63" s="12" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="I64" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J64" s="8" t="inlineStr">
@@ -2747,7 +2747,7 @@
       </c>
       <c r="I65" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J65" s="12" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="I66" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J66" s="8" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="I67" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J67" s="12" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="I68" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J68" s="8" t="inlineStr">
@@ -2907,7 +2907,7 @@
       </c>
       <c r="I69" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J69" s="12" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="I70" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J70" s="8" t="inlineStr">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="I71" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J71" s="12" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="I72" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J72" s="8" t="inlineStr">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="I73" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J73" s="12" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="I74" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J74" s="8" t="inlineStr">
@@ -3147,7 +3147,7 @@
       </c>
       <c r="I75" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J75" s="12" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="I76" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J76" s="8" t="inlineStr">
@@ -3227,7 +3227,7 @@
       </c>
       <c r="I77" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J77" s="12" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="I78" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J78" s="8" t="inlineStr">
@@ -3307,7 +3307,7 @@
       </c>
       <c r="I79" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J79" s="12" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="I80" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J80" s="8" t="inlineStr">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="I81" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J81" s="12" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="I82" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J82" s="8" t="inlineStr">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="I83" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J83" s="12" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="I84" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J84" s="8" t="inlineStr">
@@ -3547,7 +3547,7 @@
       </c>
       <c r="I85" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J85" s="12" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="I86" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J86" s="8" t="inlineStr">
@@ -3627,7 +3627,7 @@
       </c>
       <c r="I87" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J87" s="12" t="inlineStr">
@@ -3667,7 +3667,7 @@
       </c>
       <c r="I88" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J88" s="8" t="inlineStr">
@@ -3707,7 +3707,7 @@
       </c>
       <c r="I89" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J89" s="12" t="inlineStr">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="I90" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J90" s="8" t="inlineStr">
@@ -3787,7 +3787,7 @@
       </c>
       <c r="I91" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J91" s="12" t="inlineStr">
@@ -3827,7 +3827,7 @@
       </c>
       <c r="I92" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J92" s="8" t="inlineStr">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="I93" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J93" s="12" t="inlineStr">
@@ -3907,7 +3907,7 @@
       </c>
       <c r="I94" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J94" s="8" t="inlineStr">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="I95" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J95" s="12" t="inlineStr">
@@ -3987,7 +3987,7 @@
       </c>
       <c r="I96" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J96" s="8" t="inlineStr">
@@ -4027,7 +4027,7 @@
       </c>
       <c r="I97" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J97" s="12" t="inlineStr">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="I98" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J98" s="8" t="inlineStr">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="I99" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J99" s="12" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="I100" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J100" s="8" t="inlineStr">
@@ -4187,7 +4187,7 @@
       </c>
       <c r="I101" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J101" s="12" t="inlineStr">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="I102" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J102" s="8" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="I103" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J103" s="12" t="inlineStr">
@@ -4307,7 +4307,7 @@
       </c>
       <c r="I104" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J104" s="8" t="inlineStr">
@@ -4347,7 +4347,7 @@
       </c>
       <c r="I105" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J105" s="12" t="inlineStr">
@@ -4387,7 +4387,7 @@
       </c>
       <c r="I106" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J106" s="8" t="inlineStr">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="I107" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J107" s="12" t="inlineStr">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="I108" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J108" s="8" t="inlineStr">
@@ -4507,7 +4507,7 @@
       </c>
       <c r="I109" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J109" s="12" t="inlineStr">
@@ -4547,7 +4547,7 @@
       </c>
       <c r="I110" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J110" s="8" t="inlineStr">
@@ -4587,7 +4587,7 @@
       </c>
       <c r="I111" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J111" s="12" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="I112" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J112" s="8" t="inlineStr">
@@ -4667,7 +4667,7 @@
       </c>
       <c r="I113" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J113" s="12" t="inlineStr">
@@ -4707,7 +4707,7 @@
       </c>
       <c r="I114" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J114" s="8" t="inlineStr">
@@ -4747,7 +4747,7 @@
       </c>
       <c r="I115" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J115" s="12" t="inlineStr">
@@ -4787,7 +4787,7 @@
       </c>
       <c r="I116" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J116" s="8" t="inlineStr">
@@ -4827,7 +4827,7 @@
       </c>
       <c r="I117" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J117" s="12" t="inlineStr">
@@ -4867,7 +4867,7 @@
       </c>
       <c r="I118" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J118" s="8" t="inlineStr">
@@ -4907,7 +4907,7 @@
       </c>
       <c r="I119" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J119" s="12" t="inlineStr">
@@ -4947,7 +4947,7 @@
       </c>
       <c r="I120" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J120" s="8" t="inlineStr">
@@ -4987,7 +4987,7 @@
       </c>
       <c r="I121" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J121" s="12" t="inlineStr">
@@ -5027,7 +5027,7 @@
       </c>
       <c r="I122" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J122" s="8" t="inlineStr">
@@ -5067,7 +5067,7 @@
       </c>
       <c r="I123" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J123" s="12" t="inlineStr">
@@ -5107,7 +5107,7 @@
       </c>
       <c r="I124" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J124" s="8" t="inlineStr">
@@ -5147,7 +5147,7 @@
       </c>
       <c r="I125" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J125" s="12" t="inlineStr">
@@ -5187,7 +5187,7 @@
       </c>
       <c r="I126" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J126" s="8" t="inlineStr">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="I127" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J127" s="12" t="inlineStr">
@@ -5267,7 +5267,7 @@
       </c>
       <c r="I128" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J128" s="8" t="inlineStr">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="I129" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J129" s="12" t="inlineStr">
@@ -5347,7 +5347,7 @@
       </c>
       <c r="I130" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J130" s="8" t="inlineStr">
@@ -5387,7 +5387,7 @@
       </c>
       <c r="I131" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J131" s="12" t="inlineStr">
@@ -5427,7 +5427,7 @@
       </c>
       <c r="I132" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J132" s="8" t="inlineStr">
@@ -5467,7 +5467,7 @@
       </c>
       <c r="I133" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J133" s="12" t="inlineStr">
@@ -5507,7 +5507,7 @@
       </c>
       <c r="I134" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J134" s="8" t="inlineStr">
@@ -5547,7 +5547,7 @@
       </c>
       <c r="I135" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J135" s="12" t="inlineStr">
@@ -5587,7 +5587,7 @@
       </c>
       <c r="I136" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J136" s="8" t="inlineStr">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="I137" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J137" s="12" t="inlineStr">
@@ -5667,7 +5667,7 @@
       </c>
       <c r="I138" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J138" s="8" t="inlineStr">
@@ -5707,7 +5707,7 @@
       </c>
       <c r="I139" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J139" s="12" t="inlineStr">
@@ -5747,7 +5747,7 @@
       </c>
       <c r="I140" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J140" s="8" t="inlineStr">
@@ -5787,7 +5787,7 @@
       </c>
       <c r="I141" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J141" s="12" t="inlineStr">
@@ -5827,7 +5827,7 @@
       </c>
       <c r="I142" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J142" s="8" t="inlineStr">
@@ -5867,7 +5867,7 @@
       </c>
       <c r="I143" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J143" s="12" t="inlineStr">
@@ -5907,7 +5907,7 @@
       </c>
       <c r="I144" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J144" s="8" t="inlineStr">
@@ -5947,7 +5947,7 @@
       </c>
       <c r="I145" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J145" s="12" t="inlineStr">
@@ -5987,7 +5987,7 @@
       </c>
       <c r="I146" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J146" s="8" t="inlineStr">
@@ -6027,7 +6027,7 @@
       </c>
       <c r="I147" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J147" s="12" t="inlineStr">
@@ -6067,7 +6067,7 @@
       </c>
       <c r="I148" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J148" s="8" t="inlineStr">
@@ -6107,7 +6107,7 @@
       </c>
       <c r="I149" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J149" s="12" t="inlineStr">
@@ -6147,7 +6147,7 @@
       </c>
       <c r="I150" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J150" s="8" t="inlineStr">
@@ -6187,7 +6187,7 @@
       </c>
       <c r="I151" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J151" s="12" t="inlineStr">
@@ -6227,7 +6227,7 @@
       </c>
       <c r="I152" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J152" s="8" t="inlineStr">
@@ -6267,7 +6267,7 @@
       </c>
       <c r="I153" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J153" s="12" t="inlineStr">
@@ -6307,7 +6307,7 @@
       </c>
       <c r="I154" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J154" s="8" t="inlineStr">
@@ -6347,7 +6347,7 @@
       </c>
       <c r="I155" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J155" s="12" t="inlineStr">
@@ -6387,7 +6387,7 @@
       </c>
       <c r="I156" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J156" s="8" t="inlineStr">
@@ -6427,7 +6427,7 @@
       </c>
       <c r="I157" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J157" s="12" t="inlineStr">
@@ -6467,7 +6467,7 @@
       </c>
       <c r="I158" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J158" s="8" t="inlineStr">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="I159" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J159" s="12" t="inlineStr">
@@ -6547,7 +6547,7 @@
       </c>
       <c r="I160" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J160" s="8" t="inlineStr">
@@ -6587,7 +6587,7 @@
       </c>
       <c r="I161" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J161" s="12" t="inlineStr">
@@ -6627,7 +6627,7 @@
       </c>
       <c r="I162" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J162" s="8" t="inlineStr">
@@ -6667,7 +6667,7 @@
       </c>
       <c r="I163" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J163" s="12" t="inlineStr">
@@ -6707,7 +6707,7 @@
       </c>
       <c r="I164" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J164" s="8" t="inlineStr">
@@ -6747,7 +6747,7 @@
       </c>
       <c r="I165" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J165" s="12" t="inlineStr">
@@ -6787,7 +6787,7 @@
       </c>
       <c r="I166" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J166" s="8" t="inlineStr">
@@ -6827,7 +6827,7 @@
       </c>
       <c r="I167" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J167" s="12" t="inlineStr">
@@ -6867,7 +6867,7 @@
       </c>
       <c r="I168" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J168" s="8" t="inlineStr">
@@ -6907,7 +6907,7 @@
       </c>
       <c r="I169" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J169" s="12" t="inlineStr">
@@ -6947,7 +6947,7 @@
       </c>
       <c r="I170" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J170" s="8" t="inlineStr">
@@ -6987,7 +6987,7 @@
       </c>
       <c r="I171" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J171" s="12" t="inlineStr">
@@ -7027,7 +7027,7 @@
       </c>
       <c r="I172" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J172" s="8" t="inlineStr">
@@ -7067,7 +7067,7 @@
       </c>
       <c r="I173" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J173" s="12" t="inlineStr">
@@ -7107,7 +7107,7 @@
       </c>
       <c r="I174" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J174" s="8" t="inlineStr">
@@ -7147,7 +7147,7 @@
       </c>
       <c r="I175" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J175" s="12" t="inlineStr">
@@ -7187,7 +7187,7 @@
       </c>
       <c r="I176" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J176" s="8" t="inlineStr">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="I177" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J177" s="12" t="inlineStr">
@@ -7267,7 +7267,7 @@
       </c>
       <c r="I178" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J178" s="8" t="inlineStr">
@@ -7307,7 +7307,7 @@
       </c>
       <c r="I179" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J179" s="12" t="inlineStr">
@@ -7347,7 +7347,7 @@
       </c>
       <c r="I180" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J180" s="8" t="inlineStr">
@@ -7387,7 +7387,7 @@
       </c>
       <c r="I181" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J181" s="12" t="inlineStr">
@@ -7427,7 +7427,7 @@
       </c>
       <c r="I182" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J182" s="8" t="inlineStr">
@@ -7467,7 +7467,7 @@
       </c>
       <c r="I183" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J183" s="12" t="inlineStr">
@@ -7507,7 +7507,7 @@
       </c>
       <c r="I184" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J184" s="8" t="inlineStr">
@@ -7547,7 +7547,7 @@
       </c>
       <c r="I185" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J185" s="12" t="inlineStr">
@@ -7587,7 +7587,7 @@
       </c>
       <c r="I186" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J186" s="8" t="inlineStr">
@@ -7627,7 +7627,7 @@
       </c>
       <c r="I187" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J187" s="12" t="inlineStr">
@@ -7667,7 +7667,7 @@
       </c>
       <c r="I188" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J188" s="8" t="inlineStr">
@@ -7707,7 +7707,7 @@
       </c>
       <c r="I189" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J189" s="12" t="inlineStr">
@@ -7747,7 +7747,7 @@
       </c>
       <c r="I190" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J190" s="8" t="inlineStr">
@@ -7787,7 +7787,7 @@
       </c>
       <c r="I191" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J191" s="12" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="I192" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J192" s="8" t="inlineStr">
@@ -7867,7 +7867,7 @@
       </c>
       <c r="I193" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J193" s="12" t="inlineStr">
@@ -7907,7 +7907,7 @@
       </c>
       <c r="I194" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J194" s="8" t="inlineStr">
@@ -7947,7 +7947,7 @@
       </c>
       <c r="I195" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J195" s="12" t="inlineStr">
@@ -7987,7 +7987,7 @@
       </c>
       <c r="I196" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J196" s="8" t="inlineStr">
@@ -8027,7 +8027,7 @@
       </c>
       <c r="I197" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J197" s="12" t="inlineStr">
@@ -8067,7 +8067,7 @@
       </c>
       <c r="I198" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J198" s="8" t="inlineStr">
@@ -8107,7 +8107,7 @@
       </c>
       <c r="I199" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J199" s="12" t="inlineStr">
@@ -8147,7 +8147,7 @@
       </c>
       <c r="I200" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J200" s="8" t="inlineStr">
@@ -8187,7 +8187,7 @@
       </c>
       <c r="I201" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J201" s="12" t="inlineStr">
@@ -8227,7 +8227,7 @@
       </c>
       <c r="I202" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J202" s="8" t="inlineStr">
@@ -8267,7 +8267,7 @@
       </c>
       <c r="I203" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J203" s="12" t="inlineStr">
@@ -8307,7 +8307,7 @@
       </c>
       <c r="I204" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J204" s="8" t="inlineStr">
@@ -8347,7 +8347,7 @@
       </c>
       <c r="I205" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J205" s="12" t="inlineStr">
@@ -8387,7 +8387,7 @@
       </c>
       <c r="I206" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J206" s="8" t="inlineStr">
@@ -8427,7 +8427,7 @@
       </c>
       <c r="I207" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J207" s="12" t="inlineStr">
@@ -8467,7 +8467,7 @@
       </c>
       <c r="I208" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J208" s="8" t="inlineStr">
@@ -8507,7 +8507,7 @@
       </c>
       <c r="I209" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J209" s="12" t="inlineStr">
@@ -8547,7 +8547,7 @@
       </c>
       <c r="I210" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J210" s="8" t="inlineStr">
@@ -8587,7 +8587,7 @@
       </c>
       <c r="I211" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J211" s="12" t="inlineStr">
@@ -8627,7 +8627,7 @@
       </c>
       <c r="I212" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J212" s="8" t="inlineStr">
@@ -8667,7 +8667,7 @@
       </c>
       <c r="I213" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J213" s="12" t="inlineStr">
@@ -8707,7 +8707,7 @@
       </c>
       <c r="I214" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J214" s="8" t="inlineStr">
@@ -8747,7 +8747,7 @@
       </c>
       <c r="I215" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J215" s="12" t="inlineStr">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="I216" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J216" s="8" t="inlineStr">
@@ -8827,7 +8827,7 @@
       </c>
       <c r="I217" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J217" s="12" t="inlineStr">
@@ -8867,7 +8867,7 @@
       </c>
       <c r="I218" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J218" s="8" t="inlineStr">
@@ -8907,7 +8907,7 @@
       </c>
       <c r="I219" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J219" s="12" t="inlineStr">
@@ -8947,7 +8947,7 @@
       </c>
       <c r="I220" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J220" s="8" t="inlineStr">
@@ -8987,7 +8987,7 @@
       </c>
       <c r="I221" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J221" s="12" t="inlineStr">
@@ -9027,7 +9027,7 @@
       </c>
       <c r="I222" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J222" s="8" t="inlineStr">
@@ -9067,7 +9067,7 @@
       </c>
       <c r="I223" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J223" s="12" t="inlineStr">
@@ -9107,7 +9107,7 @@
       </c>
       <c r="I224" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J224" s="8" t="inlineStr">
@@ -9147,7 +9147,7 @@
       </c>
       <c r="I225" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J225" s="12" t="inlineStr">
@@ -9187,7 +9187,7 @@
       </c>
       <c r="I226" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J226" s="8" t="inlineStr">
@@ -9227,7 +9227,7 @@
       </c>
       <c r="I227" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J227" s="12" t="inlineStr">
@@ -9267,7 +9267,7 @@
       </c>
       <c r="I228" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J228" s="8" t="inlineStr">
@@ -9307,7 +9307,7 @@
       </c>
       <c r="I229" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J229" s="12" t="inlineStr">
@@ -9347,7 +9347,7 @@
       </c>
       <c r="I230" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J230" s="8" t="inlineStr">
@@ -9387,7 +9387,7 @@
       </c>
       <c r="I231" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J231" s="12" t="inlineStr">
@@ -9427,7 +9427,7 @@
       </c>
       <c r="I232" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J232" s="8" t="inlineStr">
@@ -9467,7 +9467,7 @@
       </c>
       <c r="I233" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J233" s="12" t="inlineStr">
@@ -9507,7 +9507,7 @@
       </c>
       <c r="I234" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J234" s="8" t="inlineStr">
@@ -9547,7 +9547,7 @@
       </c>
       <c r="I235" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J235" s="12" t="inlineStr">
@@ -9587,7 +9587,7 @@
       </c>
       <c r="I236" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J236" s="8" t="inlineStr">
@@ -9627,7 +9627,7 @@
       </c>
       <c r="I237" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J237" s="12" t="inlineStr">
@@ -9667,7 +9667,7 @@
       </c>
       <c r="I238" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J238" s="8" t="inlineStr">
@@ -9707,7 +9707,7 @@
       </c>
       <c r="I239" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J239" s="12" t="inlineStr">
@@ -9747,7 +9747,7 @@
       </c>
       <c r="I240" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J240" s="8" t="inlineStr">
@@ -9787,7 +9787,7 @@
       </c>
       <c r="I241" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J241" s="12" t="inlineStr">
@@ -9827,7 +9827,7 @@
       </c>
       <c r="I242" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J242" s="8" t="inlineStr">
@@ -9867,7 +9867,7 @@
       </c>
       <c r="I243" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J243" s="12" t="inlineStr">
@@ -9907,7 +9907,7 @@
       </c>
       <c r="I244" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J244" s="8" t="inlineStr">
@@ -9947,7 +9947,7 @@
       </c>
       <c r="I245" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J245" s="12" t="inlineStr">
@@ -9987,7 +9987,7 @@
       </c>
       <c r="I246" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J246" s="8" t="inlineStr">
@@ -10027,7 +10027,7 @@
       </c>
       <c r="I247" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J247" s="12" t="inlineStr">
@@ -10067,7 +10067,7 @@
       </c>
       <c r="I248" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J248" s="8" t="inlineStr">
@@ -10107,7 +10107,7 @@
       </c>
       <c r="I249" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J249" s="12" t="inlineStr">
@@ -10147,7 +10147,7 @@
       </c>
       <c r="I250" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J250" s="8" t="inlineStr">
@@ -10187,7 +10187,7 @@
       </c>
       <c r="I251" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J251" s="12" t="inlineStr">
@@ -10227,7 +10227,7 @@
       </c>
       <c r="I252" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J252" s="8" t="inlineStr">
@@ -10267,7 +10267,7 @@
       </c>
       <c r="I253" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J253" s="12" t="inlineStr">
@@ -10307,7 +10307,7 @@
       </c>
       <c r="I254" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J254" s="8" t="inlineStr">
@@ -10347,7 +10347,7 @@
       </c>
       <c r="I255" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J255" s="12" t="inlineStr">
@@ -10387,7 +10387,7 @@
       </c>
       <c r="I256" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J256" s="8" t="inlineStr">
@@ -10427,7 +10427,7 @@
       </c>
       <c r="I257" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J257" s="12" t="inlineStr">
@@ -10467,7 +10467,7 @@
       </c>
       <c r="I258" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J258" s="8" t="inlineStr">
@@ -10507,7 +10507,7 @@
       </c>
       <c r="I259" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J259" s="12" t="inlineStr">
@@ -10547,7 +10547,7 @@
       </c>
       <c r="I260" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J260" s="8" t="inlineStr">
@@ -10587,7 +10587,7 @@
       </c>
       <c r="I261" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J261" s="12" t="inlineStr">
@@ -10627,7 +10627,7 @@
       </c>
       <c r="I262" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J262" s="8" t="inlineStr">
@@ -10667,7 +10667,7 @@
       </c>
       <c r="I263" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J263" s="12" t="inlineStr">
@@ -10707,7 +10707,7 @@
       </c>
       <c r="I264" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J264" s="8" t="inlineStr">
@@ -10747,7 +10747,7 @@
       </c>
       <c r="I265" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J265" s="12" t="inlineStr">
@@ -10787,7 +10787,7 @@
       </c>
       <c r="I266" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J266" s="8" t="inlineStr">
@@ -10827,7 +10827,7 @@
       </c>
       <c r="I267" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J267" s="12" t="inlineStr">
@@ -10867,7 +10867,7 @@
       </c>
       <c r="I268" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J268" s="8" t="inlineStr">
@@ -10907,7 +10907,7 @@
       </c>
       <c r="I269" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J269" s="12" t="inlineStr">
@@ -10947,7 +10947,7 @@
       </c>
       <c r="I270" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J270" s="8" t="inlineStr">
@@ -10987,7 +10987,7 @@
       </c>
       <c r="I271" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J271" s="12" t="inlineStr">
@@ -11027,7 +11027,7 @@
       </c>
       <c r="I272" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J272" s="8" t="inlineStr">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="I273" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J273" s="12" t="inlineStr">
@@ -11107,7 +11107,7 @@
       </c>
       <c r="I274" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J274" s="8" t="inlineStr">
@@ -11147,7 +11147,7 @@
       </c>
       <c r="I275" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J275" s="12" t="inlineStr">
@@ -11187,7 +11187,7 @@
       </c>
       <c r="I276" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J276" s="8" t="inlineStr">
@@ -11227,7 +11227,7 @@
       </c>
       <c r="I277" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J277" s="12" t="inlineStr">
@@ -11267,7 +11267,7 @@
       </c>
       <c r="I278" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J278" s="8" t="inlineStr">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="I279" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J279" s="12" t="inlineStr">
@@ -11347,7 +11347,7 @@
       </c>
       <c r="I280" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J280" s="8" t="inlineStr">
@@ -11387,7 +11387,7 @@
       </c>
       <c r="I281" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J281" s="12" t="inlineStr">
@@ -11427,7 +11427,7 @@
       </c>
       <c r="I282" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J282" s="8" t="inlineStr">
@@ -11467,7 +11467,7 @@
       </c>
       <c r="I283" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J283" s="12" t="inlineStr">
@@ -11507,7 +11507,7 @@
       </c>
       <c r="I284" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J284" s="8" t="inlineStr">
@@ -11547,7 +11547,7 @@
       </c>
       <c r="I285" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J285" s="12" t="inlineStr">
@@ -11587,7 +11587,7 @@
       </c>
       <c r="I286" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J286" s="8" t="inlineStr">
@@ -11627,7 +11627,7 @@
       </c>
       <c r="I287" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J287" s="12" t="inlineStr">
@@ -11667,7 +11667,7 @@
       </c>
       <c r="I288" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J288" s="8" t="inlineStr">
@@ -11707,7 +11707,7 @@
       </c>
       <c r="I289" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J289" s="12" t="inlineStr">
@@ -11747,7 +11747,7 @@
       </c>
       <c r="I290" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J290" s="8" t="inlineStr">
@@ -11787,7 +11787,7 @@
       </c>
       <c r="I291" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J291" s="12" t="inlineStr">
@@ -11827,7 +11827,7 @@
       </c>
       <c r="I292" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J292" s="8" t="inlineStr">
@@ -11867,7 +11867,7 @@
       </c>
       <c r="I293" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J293" s="12" t="inlineStr">
@@ -11907,7 +11907,7 @@
       </c>
       <c r="I294" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J294" s="8" t="inlineStr">
@@ -11947,7 +11947,7 @@
       </c>
       <c r="I295" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J295" s="12" t="inlineStr">
@@ -11987,7 +11987,7 @@
       </c>
       <c r="I296" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J296" s="8" t="inlineStr">
@@ -12027,7 +12027,7 @@
       </c>
       <c r="I297" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J297" s="12" t="inlineStr">
@@ -12067,7 +12067,7 @@
       </c>
       <c r="I298" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J298" s="8" t="inlineStr">
@@ -12107,7 +12107,7 @@
       </c>
       <c r="I299" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J299" s="12" t="inlineStr">
@@ -12147,7 +12147,7 @@
       </c>
       <c r="I300" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J300" s="8" t="inlineStr">
@@ -12187,7 +12187,7 @@
       </c>
       <c r="I301" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J301" s="12" t="inlineStr">
@@ -12227,7 +12227,7 @@
       </c>
       <c r="I302" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J302" s="8" t="inlineStr">
@@ -12267,7 +12267,7 @@
       </c>
       <c r="I303" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J303" s="12" t="inlineStr">
@@ -12307,7 +12307,7 @@
       </c>
       <c r="I304" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J304" s="8" t="inlineStr">
@@ -12347,7 +12347,7 @@
       </c>
       <c r="I305" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J305" s="12" t="inlineStr">
@@ -12387,7 +12387,7 @@
       </c>
       <c r="I306" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J306" s="8" t="inlineStr">
@@ -12427,7 +12427,7 @@
       </c>
       <c r="I307" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J307" s="12" t="inlineStr">
@@ -12467,7 +12467,7 @@
       </c>
       <c r="I308" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J308" s="8" t="inlineStr">
@@ -12507,7 +12507,7 @@
       </c>
       <c r="I309" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J309" s="12" t="inlineStr">
@@ -12547,7 +12547,7 @@
       </c>
       <c r="I310" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J310" s="8" t="inlineStr">
@@ -12587,7 +12587,7 @@
       </c>
       <c r="I311" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J311" s="12" t="inlineStr">
@@ -12627,7 +12627,7 @@
       </c>
       <c r="I312" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J312" s="8" t="inlineStr">
@@ -12667,7 +12667,7 @@
       </c>
       <c r="I313" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J313" s="12" t="inlineStr">
@@ -12707,7 +12707,7 @@
       </c>
       <c r="I314" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J314" s="8" t="inlineStr">
@@ -12747,7 +12747,7 @@
       </c>
       <c r="I315" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J315" s="12" t="inlineStr">
@@ -12787,7 +12787,7 @@
       </c>
       <c r="I316" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J316" s="8" t="inlineStr">
@@ -12827,7 +12827,7 @@
       </c>
       <c r="I317" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J317" s="12" t="inlineStr">
@@ -12867,7 +12867,7 @@
       </c>
       <c r="I318" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J318" s="8" t="inlineStr">
@@ -12907,7 +12907,7 @@
       </c>
       <c r="I319" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J319" s="12" t="inlineStr">
@@ -12947,7 +12947,7 @@
       </c>
       <c r="I320" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J320" s="8" t="inlineStr">
@@ -12987,7 +12987,7 @@
       </c>
       <c r="I321" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J321" s="12" t="inlineStr">
@@ -13027,7 +13027,7 @@
       </c>
       <c r="I322" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J322" s="8" t="inlineStr">
@@ -13067,7 +13067,7 @@
       </c>
       <c r="I323" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J323" s="12" t="inlineStr">
@@ -13107,7 +13107,7 @@
       </c>
       <c r="I324" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J324" s="8" t="inlineStr">
@@ -13147,7 +13147,7 @@
       </c>
       <c r="I325" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J325" s="12" t="inlineStr">
@@ -13187,7 +13187,7 @@
       </c>
       <c r="I326" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J326" s="8" t="inlineStr">
@@ -13227,7 +13227,7 @@
       </c>
       <c r="I327" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J327" s="12" t="inlineStr">
@@ -13267,7 +13267,7 @@
       </c>
       <c r="I328" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J328" s="8" t="inlineStr">
@@ -13307,7 +13307,7 @@
       </c>
       <c r="I329" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J329" s="12" t="inlineStr">
@@ -13347,7 +13347,7 @@
       </c>
       <c r="I330" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J330" s="8" t="inlineStr">
@@ -13387,7 +13387,7 @@
       </c>
       <c r="I331" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J331" s="12" t="inlineStr">
@@ -13427,7 +13427,7 @@
       </c>
       <c r="I332" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J332" s="8" t="inlineStr">
@@ -13467,7 +13467,7 @@
       </c>
       <c r="I333" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J333" s="12" t="inlineStr">
@@ -13507,7 +13507,7 @@
       </c>
       <c r="I334" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J334" s="8" t="inlineStr">
@@ -13547,7 +13547,7 @@
       </c>
       <c r="I335" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J335" s="12" t="inlineStr">
@@ -13587,7 +13587,7 @@
       </c>
       <c r="I336" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J336" s="8" t="inlineStr">
@@ -13627,7 +13627,7 @@
       </c>
       <c r="I337" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J337" s="12" t="inlineStr">
@@ -13667,7 +13667,7 @@
       </c>
       <c r="I338" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J338" s="8" t="inlineStr">
@@ -13707,7 +13707,7 @@
       </c>
       <c r="I339" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J339" s="12" t="inlineStr">
@@ -13747,7 +13747,7 @@
       </c>
       <c r="I340" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J340" s="8" t="inlineStr">
@@ -13787,7 +13787,7 @@
       </c>
       <c r="I341" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J341" s="12" t="inlineStr">
@@ -13827,7 +13827,7 @@
       </c>
       <c r="I342" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J342" s="8" t="inlineStr">
@@ -13867,7 +13867,7 @@
       </c>
       <c r="I343" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J343" s="12" t="inlineStr">
@@ -13907,7 +13907,7 @@
       </c>
       <c r="I344" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J344" s="8" t="inlineStr">
@@ -13947,7 +13947,7 @@
       </c>
       <c r="I345" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J345" s="12" t="inlineStr">
@@ -13987,7 +13987,7 @@
       </c>
       <c r="I346" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J346" s="8" t="inlineStr">
@@ -14027,7 +14027,7 @@
       </c>
       <c r="I347" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J347" s="12" t="inlineStr">
@@ -14067,7 +14067,7 @@
       </c>
       <c r="I348" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J348" s="8" t="inlineStr">
@@ -14107,7 +14107,7 @@
       </c>
       <c r="I349" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J349" s="12" t="inlineStr">
@@ -14147,7 +14147,7 @@
       </c>
       <c r="I350" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J350" s="8" t="inlineStr">
@@ -14187,7 +14187,7 @@
       </c>
       <c r="I351" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J351" s="12" t="inlineStr">
@@ -14227,7 +14227,7 @@
       </c>
       <c r="I352" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J352" s="8" t="inlineStr">
@@ -14267,7 +14267,7 @@
       </c>
       <c r="I353" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J353" s="12" t="inlineStr">
@@ -14307,7 +14307,7 @@
       </c>
       <c r="I354" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J354" s="8" t="inlineStr">
@@ -14347,7 +14347,7 @@
       </c>
       <c r="I355" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J355" s="12" t="inlineStr">
@@ -14387,7 +14387,7 @@
       </c>
       <c r="I356" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J356" s="8" t="inlineStr">
@@ -14427,7 +14427,7 @@
       </c>
       <c r="I357" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J357" s="12" t="inlineStr">
@@ -14467,7 +14467,7 @@
       </c>
       <c r="I358" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J358" s="8" t="inlineStr">
@@ -14507,7 +14507,7 @@
       </c>
       <c r="I359" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J359" s="12" t="inlineStr">
@@ -14547,7 +14547,7 @@
       </c>
       <c r="I360" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J360" s="8" t="inlineStr">
@@ -14587,7 +14587,7 @@
       </c>
       <c r="I361" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J361" s="12" t="inlineStr">
@@ -14627,7 +14627,7 @@
       </c>
       <c r="I362" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J362" s="8" t="inlineStr">
@@ -14667,7 +14667,7 @@
       </c>
       <c r="I363" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J363" s="12" t="inlineStr">
@@ -14707,7 +14707,7 @@
       </c>
       <c r="I364" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J364" s="8" t="inlineStr">
@@ -14747,7 +14747,7 @@
       </c>
       <c r="I365" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J365" s="12" t="inlineStr">
@@ -14787,7 +14787,7 @@
       </c>
       <c r="I366" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J366" s="8" t="inlineStr">
@@ -14827,7 +14827,7 @@
       </c>
       <c r="I367" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J367" s="12" t="inlineStr">
@@ -14867,7 +14867,7 @@
       </c>
       <c r="I368" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J368" s="8" t="inlineStr">
@@ -14907,7 +14907,7 @@
       </c>
       <c r="I369" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J369" s="12" t="inlineStr">
@@ -14947,7 +14947,7 @@
       </c>
       <c r="I370" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J370" s="8" t="inlineStr">
@@ -14987,7 +14987,7 @@
       </c>
       <c r="I371" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J371" s="12" t="inlineStr">
@@ -15027,7 +15027,7 @@
       </c>
       <c r="I372" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J372" s="8" t="inlineStr">
@@ -15067,7 +15067,7 @@
       </c>
       <c r="I373" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J373" s="12" t="inlineStr">
@@ -15107,7 +15107,7 @@
       </c>
       <c r="I374" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J374" s="8" t="inlineStr">
@@ -15147,7 +15147,7 @@
       </c>
       <c r="I375" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J375" s="12" t="inlineStr">
@@ -15187,7 +15187,7 @@
       </c>
       <c r="I376" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J376" s="8" t="inlineStr">
@@ -15227,7 +15227,7 @@
       </c>
       <c r="I377" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J377" s="12" t="inlineStr">
@@ -15267,7 +15267,7 @@
       </c>
       <c r="I378" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J378" s="8" t="inlineStr">
@@ -15307,7 +15307,7 @@
       </c>
       <c r="I379" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J379" s="12" t="inlineStr">
@@ -15347,7 +15347,7 @@
       </c>
       <c r="I380" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J380" s="8" t="inlineStr">
@@ -15387,7 +15387,7 @@
       </c>
       <c r="I381" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J381" s="12" t="inlineStr">
@@ -15427,7 +15427,7 @@
       </c>
       <c r="I382" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J382" s="8" t="inlineStr">
@@ -15467,7 +15467,7 @@
       </c>
       <c r="I383" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J383" s="12" t="inlineStr">
@@ -15507,7 +15507,7 @@
       </c>
       <c r="I384" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J384" s="8" t="inlineStr">
@@ -15547,7 +15547,7 @@
       </c>
       <c r="I385" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J385" s="12" t="inlineStr">
@@ -15587,7 +15587,7 @@
       </c>
       <c r="I386" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J386" s="8" t="inlineStr">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="I387" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J387" s="12" t="inlineStr">
@@ -15667,7 +15667,7 @@
       </c>
       <c r="I388" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J388" s="8" t="inlineStr">
@@ -15707,7 +15707,7 @@
       </c>
       <c r="I389" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J389" s="12" t="inlineStr">
@@ -15747,7 +15747,7 @@
       </c>
       <c r="I390" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J390" s="8" t="inlineStr">
@@ -15787,7 +15787,7 @@
       </c>
       <c r="I391" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J391" s="12" t="inlineStr">
@@ -15827,7 +15827,7 @@
       </c>
       <c r="I392" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J392" s="8" t="inlineStr">
@@ -15867,7 +15867,7 @@
       </c>
       <c r="I393" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J393" s="12" t="inlineStr">
@@ -15907,7 +15907,7 @@
       </c>
       <c r="I394" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J394" s="8" t="inlineStr">
@@ -15947,7 +15947,7 @@
       </c>
       <c r="I395" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J395" s="12" t="inlineStr">
@@ -15987,7 +15987,7 @@
       </c>
       <c r="I396" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J396" s="8" t="inlineStr">
@@ -16027,7 +16027,7 @@
       </c>
       <c r="I397" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J397" s="12" t="inlineStr">
@@ -16067,7 +16067,7 @@
       </c>
       <c r="I398" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J398" s="8" t="inlineStr">
@@ -16107,7 +16107,7 @@
       </c>
       <c r="I399" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J399" s="12" t="inlineStr">
@@ -16147,7 +16147,7 @@
       </c>
       <c r="I400" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J400" s="8" t="inlineStr">
@@ -16187,7 +16187,7 @@
       </c>
       <c r="I401" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J401" s="12" t="inlineStr">
@@ -16227,7 +16227,7 @@
       </c>
       <c r="I402" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J402" s="8" t="inlineStr">
@@ -16267,7 +16267,7 @@
       </c>
       <c r="I403" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J403" s="12" t="inlineStr">
@@ -16307,7 +16307,7 @@
       </c>
       <c r="I404" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J404" s="8" t="inlineStr">
@@ -16347,7 +16347,7 @@
       </c>
       <c r="I405" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J405" s="12" t="inlineStr">
@@ -16387,7 +16387,7 @@
       </c>
       <c r="I406" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J406" s="8" t="inlineStr">
@@ -16427,7 +16427,7 @@
       </c>
       <c r="I407" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J407" s="12" t="inlineStr">
@@ -16467,7 +16467,7 @@
       </c>
       <c r="I408" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J408" s="8" t="inlineStr">
@@ -16507,7 +16507,7 @@
       </c>
       <c r="I409" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J409" s="12" t="inlineStr">
@@ -16547,7 +16547,7 @@
       </c>
       <c r="I410" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J410" s="8" t="inlineStr">
@@ -16587,7 +16587,7 @@
       </c>
       <c r="I411" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J411" s="12" t="inlineStr">
@@ -16627,7 +16627,7 @@
       </c>
       <c r="I412" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J412" s="8" t="inlineStr">
@@ -16667,7 +16667,7 @@
       </c>
       <c r="I413" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J413" s="12" t="inlineStr">
@@ -16707,7 +16707,7 @@
       </c>
       <c r="I414" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J414" s="8" t="inlineStr">
@@ -16747,7 +16747,7 @@
       </c>
       <c r="I415" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J415" s="12" t="inlineStr">
@@ -16787,7 +16787,7 @@
       </c>
       <c r="I416" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J416" s="8" t="inlineStr">
@@ -16827,7 +16827,7 @@
       </c>
       <c r="I417" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J417" s="12" t="inlineStr">
@@ -16867,7 +16867,7 @@
       </c>
       <c r="I418" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J418" s="8" t="inlineStr">
@@ -16907,7 +16907,7 @@
       </c>
       <c r="I419" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J419" s="12" t="inlineStr">
@@ -16947,7 +16947,7 @@
       </c>
       <c r="I420" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J420" s="8" t="inlineStr">
@@ -16987,7 +16987,7 @@
       </c>
       <c r="I421" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J421" s="12" t="inlineStr">
@@ -17027,7 +17027,7 @@
       </c>
       <c r="I422" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J422" s="8" t="inlineStr">
@@ -17067,7 +17067,7 @@
       </c>
       <c r="I423" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J423" s="12" t="inlineStr">
@@ -17107,7 +17107,7 @@
       </c>
       <c r="I424" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J424" s="8" t="inlineStr">
@@ -17147,7 +17147,7 @@
       </c>
       <c r="I425" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J425" s="12" t="inlineStr">
@@ -17187,7 +17187,7 @@
       </c>
       <c r="I426" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J426" s="8" t="inlineStr">
@@ -17227,7 +17227,7 @@
       </c>
       <c r="I427" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J427" s="12" t="inlineStr">
@@ -17267,7 +17267,7 @@
       </c>
       <c r="I428" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J428" s="8" t="inlineStr">
@@ -17307,7 +17307,7 @@
       </c>
       <c r="I429" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J429" s="12" t="inlineStr">
@@ -17347,7 +17347,7 @@
       </c>
       <c r="I430" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J430" s="8" t="inlineStr">
@@ -17387,7 +17387,7 @@
       </c>
       <c r="I431" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J431" s="12" t="inlineStr">
@@ -17427,7 +17427,7 @@
       </c>
       <c r="I432" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J432" s="8" t="inlineStr">
@@ -17467,7 +17467,7 @@
       </c>
       <c r="I433" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J433" s="12" t="inlineStr">
@@ -17507,7 +17507,7 @@
       </c>
       <c r="I434" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J434" s="8" t="inlineStr">
@@ -17547,7 +17547,7 @@
       </c>
       <c r="I435" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J435" s="12" t="inlineStr">
@@ -17587,7 +17587,7 @@
       </c>
       <c r="I436" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J436" s="8" t="inlineStr">
@@ -17627,7 +17627,7 @@
       </c>
       <c r="I437" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J437" s="12" t="inlineStr">
@@ -17667,7 +17667,7 @@
       </c>
       <c r="I438" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J438" s="8" t="inlineStr">
@@ -17707,7 +17707,7 @@
       </c>
       <c r="I439" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J439" s="12" t="inlineStr">
@@ -17747,7 +17747,7 @@
       </c>
       <c r="I440" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J440" s="8" t="inlineStr">
@@ -17787,7 +17787,7 @@
       </c>
       <c r="I441" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J441" s="12" t="inlineStr">
@@ -17827,7 +17827,7 @@
       </c>
       <c r="I442" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J442" s="8" t="inlineStr">
@@ -17867,7 +17867,7 @@
       </c>
       <c r="I443" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J443" s="12" t="inlineStr">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="I444" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J444" s="8" t="inlineStr">
@@ -17947,7 +17947,7 @@
       </c>
       <c r="I445" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J445" s="12" t="inlineStr">
@@ -17987,7 +17987,7 @@
       </c>
       <c r="I446" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J446" s="8" t="inlineStr">
@@ -18027,7 +18027,7 @@
       </c>
       <c r="I447" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J447" s="12" t="inlineStr">
@@ -18067,7 +18067,7 @@
       </c>
       <c r="I448" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J448" s="8" t="inlineStr">
@@ -18107,7 +18107,7 @@
       </c>
       <c r="I449" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J449" s="12" t="inlineStr">
@@ -18147,7 +18147,7 @@
       </c>
       <c r="I450" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J450" s="8" t="inlineStr">
@@ -18187,7 +18187,7 @@
       </c>
       <c r="I451" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J451" s="12" t="inlineStr">
@@ -18227,7 +18227,7 @@
       </c>
       <c r="I452" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J452" s="8" t="inlineStr">
@@ -18267,7 +18267,7 @@
       </c>
       <c r="I453" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J453" s="12" t="inlineStr">
@@ -18307,7 +18307,7 @@
       </c>
       <c r="I454" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J454" s="8" t="inlineStr">
@@ -18347,7 +18347,7 @@
       </c>
       <c r="I455" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J455" s="12" t="inlineStr">
@@ -18387,7 +18387,7 @@
       </c>
       <c r="I456" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J456" s="8" t="inlineStr">
@@ -18427,7 +18427,7 @@
       </c>
       <c r="I457" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/reservas-internacionales/</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
         </is>
       </c>
       <c r="J457" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Ajuste visual puntual del calendario: fondo verde claro en próximas.
- Añade `background: #edf3ef` y `border-color: #dce7e1` a
  `.cal-highlights .cal-upcoming` para diferenciar el bloque izquierdo
  sin cambiar la estructura.
- Regenera datos y Excel (pipeline actualizó URL de RESERVAS al
  endpoint estable del estado de cuenta semanal).
- Actualiza el test de regresión de variaciones para el dato más
  reciente de IMFBCF (Jun 26).
- Hace el test de URL de RESERVAS tolerante a fallos de red en CI
  (mantiene la validación 404/410, omite en timeouts o errores de
  conectividad).

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/downloads/indicadores/RESERVAS/RESERVAS_datos.xlsx
+++ b/downloads/indicadores/RESERVAS/RESERVAS_datos.xlsx
@@ -510,7 +510,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>URL del boletín / serie: https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf · Fecha de publicación: —</t>
+          <t>URL del boletín / serie: https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html · Fecha de publicación: —</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J6" s="8" t="inlineStr">
@@ -627,7 +627,7 @@
       </c>
       <c r="I7" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J7" s="12" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J10" s="8" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J11" s="12" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J12" s="8" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J13" s="12" t="inlineStr">
@@ -879,7 +879,7 @@
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J14" s="8" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J16" s="8" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J17" s="12" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J18" s="8" t="inlineStr">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="I19" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J19" s="12" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J20" s="8" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="I21" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J21" s="12" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J22" s="8" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="I23" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J23" s="12" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J24" s="8" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="I25" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J25" s="12" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="I26" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J26" s="8" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="I27" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J27" s="12" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J28" s="8" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="I29" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J29" s="12" t="inlineStr">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J30" s="8" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="I31" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J31" s="12" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J32" s="8" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="I33" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J33" s="12" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J34" s="8" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="I35" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J35" s="12" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J36" s="8" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="I37" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J37" s="12" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="I38" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J38" s="8" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="I39" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J39" s="12" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="I40" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J40" s="8" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="I41" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J41" s="12" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="I42" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J42" s="8" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="I43" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J43" s="12" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="I44" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J44" s="8" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="I45" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J45" s="12" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="I46" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J46" s="8" t="inlineStr">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="I47" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J47" s="12" t="inlineStr">
@@ -2103,7 +2103,7 @@
       </c>
       <c r="I48" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J48" s="8" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="I49" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J49" s="12" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="I50" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J50" s="8" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="I51" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J51" s="12" t="inlineStr">
@@ -2247,7 +2247,7 @@
       </c>
       <c r="I52" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J52" s="8" t="inlineStr">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="I53" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J53" s="12" t="inlineStr">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="I54" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J54" s="8" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="I55" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J55" s="12" t="inlineStr">
@@ -2391,7 +2391,7 @@
       </c>
       <c r="I56" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J56" s="8" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="I57" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J57" s="12" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="I58" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J58" s="8" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="I59" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J59" s="12" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="I60" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J60" s="8" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="I61" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J61" s="12" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="I62" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J62" s="8" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="I63" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J63" s="12" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="I64" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J64" s="8" t="inlineStr">
@@ -2747,7 +2747,7 @@
       </c>
       <c r="I65" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J65" s="12" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="I66" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J66" s="8" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="I67" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J67" s="12" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="I68" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J68" s="8" t="inlineStr">
@@ -2907,7 +2907,7 @@
       </c>
       <c r="I69" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J69" s="12" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="I70" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J70" s="8" t="inlineStr">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="I71" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J71" s="12" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="I72" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J72" s="8" t="inlineStr">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="I73" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J73" s="12" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="I74" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J74" s="8" t="inlineStr">
@@ -3147,7 +3147,7 @@
       </c>
       <c r="I75" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J75" s="12" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="I76" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J76" s="8" t="inlineStr">
@@ -3227,7 +3227,7 @@
       </c>
       <c r="I77" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J77" s="12" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="I78" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J78" s="8" t="inlineStr">
@@ -3307,7 +3307,7 @@
       </c>
       <c r="I79" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J79" s="12" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="I80" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J80" s="8" t="inlineStr">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="I81" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J81" s="12" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="I82" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J82" s="8" t="inlineStr">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="I83" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J83" s="12" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="I84" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J84" s="8" t="inlineStr">
@@ -3547,7 +3547,7 @@
       </c>
       <c r="I85" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J85" s="12" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="I86" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J86" s="8" t="inlineStr">
@@ -3627,7 +3627,7 @@
       </c>
       <c r="I87" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J87" s="12" t="inlineStr">
@@ -3667,7 +3667,7 @@
       </c>
       <c r="I88" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J88" s="8" t="inlineStr">
@@ -3707,7 +3707,7 @@
       </c>
       <c r="I89" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J89" s="12" t="inlineStr">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="I90" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J90" s="8" t="inlineStr">
@@ -3787,7 +3787,7 @@
       </c>
       <c r="I91" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J91" s="12" t="inlineStr">
@@ -3827,7 +3827,7 @@
       </c>
       <c r="I92" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J92" s="8" t="inlineStr">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="I93" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J93" s="12" t="inlineStr">
@@ -3907,7 +3907,7 @@
       </c>
       <c r="I94" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J94" s="8" t="inlineStr">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="I95" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J95" s="12" t="inlineStr">
@@ -3987,7 +3987,7 @@
       </c>
       <c r="I96" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J96" s="8" t="inlineStr">
@@ -4027,7 +4027,7 @@
       </c>
       <c r="I97" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J97" s="12" t="inlineStr">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="I98" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J98" s="8" t="inlineStr">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="I99" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J99" s="12" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="I100" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J100" s="8" t="inlineStr">
@@ -4187,7 +4187,7 @@
       </c>
       <c r="I101" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J101" s="12" t="inlineStr">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="I102" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J102" s="8" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="I103" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J103" s="12" t="inlineStr">
@@ -4307,7 +4307,7 @@
       </c>
       <c r="I104" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J104" s="8" t="inlineStr">
@@ -4347,7 +4347,7 @@
       </c>
       <c r="I105" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J105" s="12" t="inlineStr">
@@ -4387,7 +4387,7 @@
       </c>
       <c r="I106" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J106" s="8" t="inlineStr">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="I107" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J107" s="12" t="inlineStr">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="I108" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J108" s="8" t="inlineStr">
@@ -4507,7 +4507,7 @@
       </c>
       <c r="I109" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J109" s="12" t="inlineStr">
@@ -4547,7 +4547,7 @@
       </c>
       <c r="I110" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J110" s="8" t="inlineStr">
@@ -4587,7 +4587,7 @@
       </c>
       <c r="I111" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J111" s="12" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="I112" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J112" s="8" t="inlineStr">
@@ -4667,7 +4667,7 @@
       </c>
       <c r="I113" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J113" s="12" t="inlineStr">
@@ -4707,7 +4707,7 @@
       </c>
       <c r="I114" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J114" s="8" t="inlineStr">
@@ -4747,7 +4747,7 @@
       </c>
       <c r="I115" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J115" s="12" t="inlineStr">
@@ -4787,7 +4787,7 @@
       </c>
       <c r="I116" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J116" s="8" t="inlineStr">
@@ -4827,7 +4827,7 @@
       </c>
       <c r="I117" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J117" s="12" t="inlineStr">
@@ -4867,7 +4867,7 @@
       </c>
       <c r="I118" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J118" s="8" t="inlineStr">
@@ -4907,7 +4907,7 @@
       </c>
       <c r="I119" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J119" s="12" t="inlineStr">
@@ -4947,7 +4947,7 @@
       </c>
       <c r="I120" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J120" s="8" t="inlineStr">
@@ -4987,7 +4987,7 @@
       </c>
       <c r="I121" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J121" s="12" t="inlineStr">
@@ -5027,7 +5027,7 @@
       </c>
       <c r="I122" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J122" s="8" t="inlineStr">
@@ -5067,7 +5067,7 @@
       </c>
       <c r="I123" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J123" s="12" t="inlineStr">
@@ -5107,7 +5107,7 @@
       </c>
       <c r="I124" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J124" s="8" t="inlineStr">
@@ -5147,7 +5147,7 @@
       </c>
       <c r="I125" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J125" s="12" t="inlineStr">
@@ -5187,7 +5187,7 @@
       </c>
       <c r="I126" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J126" s="8" t="inlineStr">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="I127" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J127" s="12" t="inlineStr">
@@ -5267,7 +5267,7 @@
       </c>
       <c r="I128" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J128" s="8" t="inlineStr">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="I129" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J129" s="12" t="inlineStr">
@@ -5347,7 +5347,7 @@
       </c>
       <c r="I130" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J130" s="8" t="inlineStr">
@@ -5387,7 +5387,7 @@
       </c>
       <c r="I131" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J131" s="12" t="inlineStr">
@@ -5427,7 +5427,7 @@
       </c>
       <c r="I132" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J132" s="8" t="inlineStr">
@@ -5467,7 +5467,7 @@
       </c>
       <c r="I133" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J133" s="12" t="inlineStr">
@@ -5507,7 +5507,7 @@
       </c>
       <c r="I134" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J134" s="8" t="inlineStr">
@@ -5547,7 +5547,7 @@
       </c>
       <c r="I135" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J135" s="12" t="inlineStr">
@@ -5587,7 +5587,7 @@
       </c>
       <c r="I136" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J136" s="8" t="inlineStr">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="I137" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J137" s="12" t="inlineStr">
@@ -5667,7 +5667,7 @@
       </c>
       <c r="I138" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J138" s="8" t="inlineStr">
@@ -5707,7 +5707,7 @@
       </c>
       <c r="I139" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J139" s="12" t="inlineStr">
@@ -5747,7 +5747,7 @@
       </c>
       <c r="I140" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J140" s="8" t="inlineStr">
@@ -5787,7 +5787,7 @@
       </c>
       <c r="I141" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J141" s="12" t="inlineStr">
@@ -5827,7 +5827,7 @@
       </c>
       <c r="I142" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J142" s="8" t="inlineStr">
@@ -5867,7 +5867,7 @@
       </c>
       <c r="I143" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J143" s="12" t="inlineStr">
@@ -5907,7 +5907,7 @@
       </c>
       <c r="I144" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J144" s="8" t="inlineStr">
@@ -5947,7 +5947,7 @@
       </c>
       <c r="I145" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J145" s="12" t="inlineStr">
@@ -5987,7 +5987,7 @@
       </c>
       <c r="I146" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J146" s="8" t="inlineStr">
@@ -6027,7 +6027,7 @@
       </c>
       <c r="I147" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J147" s="12" t="inlineStr">
@@ -6067,7 +6067,7 @@
       </c>
       <c r="I148" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J148" s="8" t="inlineStr">
@@ -6107,7 +6107,7 @@
       </c>
       <c r="I149" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J149" s="12" t="inlineStr">
@@ -6147,7 +6147,7 @@
       </c>
       <c r="I150" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J150" s="8" t="inlineStr">
@@ -6187,7 +6187,7 @@
       </c>
       <c r="I151" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J151" s="12" t="inlineStr">
@@ -6227,7 +6227,7 @@
       </c>
       <c r="I152" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J152" s="8" t="inlineStr">
@@ -6267,7 +6267,7 @@
       </c>
       <c r="I153" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J153" s="12" t="inlineStr">
@@ -6307,7 +6307,7 @@
       </c>
       <c r="I154" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J154" s="8" t="inlineStr">
@@ -6347,7 +6347,7 @@
       </c>
       <c r="I155" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J155" s="12" t="inlineStr">
@@ -6387,7 +6387,7 @@
       </c>
       <c r="I156" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J156" s="8" t="inlineStr">
@@ -6427,7 +6427,7 @@
       </c>
       <c r="I157" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J157" s="12" t="inlineStr">
@@ -6467,7 +6467,7 @@
       </c>
       <c r="I158" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J158" s="8" t="inlineStr">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="I159" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J159" s="12" t="inlineStr">
@@ -6547,7 +6547,7 @@
       </c>
       <c r="I160" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J160" s="8" t="inlineStr">
@@ -6587,7 +6587,7 @@
       </c>
       <c r="I161" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J161" s="12" t="inlineStr">
@@ -6627,7 +6627,7 @@
       </c>
       <c r="I162" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J162" s="8" t="inlineStr">
@@ -6667,7 +6667,7 @@
       </c>
       <c r="I163" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J163" s="12" t="inlineStr">
@@ -6707,7 +6707,7 @@
       </c>
       <c r="I164" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J164" s="8" t="inlineStr">
@@ -6747,7 +6747,7 @@
       </c>
       <c r="I165" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J165" s="12" t="inlineStr">
@@ -6787,7 +6787,7 @@
       </c>
       <c r="I166" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J166" s="8" t="inlineStr">
@@ -6827,7 +6827,7 @@
       </c>
       <c r="I167" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J167" s="12" t="inlineStr">
@@ -6867,7 +6867,7 @@
       </c>
       <c r="I168" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J168" s="8" t="inlineStr">
@@ -6907,7 +6907,7 @@
       </c>
       <c r="I169" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J169" s="12" t="inlineStr">
@@ -6947,7 +6947,7 @@
       </c>
       <c r="I170" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J170" s="8" t="inlineStr">
@@ -6987,7 +6987,7 @@
       </c>
       <c r="I171" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J171" s="12" t="inlineStr">
@@ -7027,7 +7027,7 @@
       </c>
       <c r="I172" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J172" s="8" t="inlineStr">
@@ -7067,7 +7067,7 @@
       </c>
       <c r="I173" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J173" s="12" t="inlineStr">
@@ -7107,7 +7107,7 @@
       </c>
       <c r="I174" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J174" s="8" t="inlineStr">
@@ -7147,7 +7147,7 @@
       </c>
       <c r="I175" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J175" s="12" t="inlineStr">
@@ -7187,7 +7187,7 @@
       </c>
       <c r="I176" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J176" s="8" t="inlineStr">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="I177" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J177" s="12" t="inlineStr">
@@ -7267,7 +7267,7 @@
       </c>
       <c r="I178" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J178" s="8" t="inlineStr">
@@ -7307,7 +7307,7 @@
       </c>
       <c r="I179" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J179" s="12" t="inlineStr">
@@ -7347,7 +7347,7 @@
       </c>
       <c r="I180" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J180" s="8" t="inlineStr">
@@ -7387,7 +7387,7 @@
       </c>
       <c r="I181" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J181" s="12" t="inlineStr">
@@ -7427,7 +7427,7 @@
       </c>
       <c r="I182" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J182" s="8" t="inlineStr">
@@ -7467,7 +7467,7 @@
       </c>
       <c r="I183" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J183" s="12" t="inlineStr">
@@ -7507,7 +7507,7 @@
       </c>
       <c r="I184" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J184" s="8" t="inlineStr">
@@ -7547,7 +7547,7 @@
       </c>
       <c r="I185" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J185" s="12" t="inlineStr">
@@ -7587,7 +7587,7 @@
       </c>
       <c r="I186" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J186" s="8" t="inlineStr">
@@ -7627,7 +7627,7 @@
       </c>
       <c r="I187" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J187" s="12" t="inlineStr">
@@ -7667,7 +7667,7 @@
       </c>
       <c r="I188" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J188" s="8" t="inlineStr">
@@ -7707,7 +7707,7 @@
       </c>
       <c r="I189" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J189" s="12" t="inlineStr">
@@ -7747,7 +7747,7 @@
       </c>
       <c r="I190" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J190" s="8" t="inlineStr">
@@ -7787,7 +7787,7 @@
       </c>
       <c r="I191" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J191" s="12" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="I192" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J192" s="8" t="inlineStr">
@@ -7867,7 +7867,7 @@
       </c>
       <c r="I193" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J193" s="12" t="inlineStr">
@@ -7907,7 +7907,7 @@
       </c>
       <c r="I194" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J194" s="8" t="inlineStr">
@@ -7947,7 +7947,7 @@
       </c>
       <c r="I195" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J195" s="12" t="inlineStr">
@@ -7987,7 +7987,7 @@
       </c>
       <c r="I196" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J196" s="8" t="inlineStr">
@@ -8027,7 +8027,7 @@
       </c>
       <c r="I197" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J197" s="12" t="inlineStr">
@@ -8067,7 +8067,7 @@
       </c>
       <c r="I198" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J198" s="8" t="inlineStr">
@@ -8107,7 +8107,7 @@
       </c>
       <c r="I199" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J199" s="12" t="inlineStr">
@@ -8147,7 +8147,7 @@
       </c>
       <c r="I200" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J200" s="8" t="inlineStr">
@@ -8187,7 +8187,7 @@
       </c>
       <c r="I201" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J201" s="12" t="inlineStr">
@@ -8227,7 +8227,7 @@
       </c>
       <c r="I202" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J202" s="8" t="inlineStr">
@@ -8267,7 +8267,7 @@
       </c>
       <c r="I203" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J203" s="12" t="inlineStr">
@@ -8307,7 +8307,7 @@
       </c>
       <c r="I204" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J204" s="8" t="inlineStr">
@@ -8347,7 +8347,7 @@
       </c>
       <c r="I205" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J205" s="12" t="inlineStr">
@@ -8387,7 +8387,7 @@
       </c>
       <c r="I206" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J206" s="8" t="inlineStr">
@@ -8427,7 +8427,7 @@
       </c>
       <c r="I207" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J207" s="12" t="inlineStr">
@@ -8467,7 +8467,7 @@
       </c>
       <c r="I208" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J208" s="8" t="inlineStr">
@@ -8507,7 +8507,7 @@
       </c>
       <c r="I209" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J209" s="12" t="inlineStr">
@@ -8547,7 +8547,7 @@
       </c>
       <c r="I210" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J210" s="8" t="inlineStr">
@@ -8587,7 +8587,7 @@
       </c>
       <c r="I211" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J211" s="12" t="inlineStr">
@@ -8627,7 +8627,7 @@
       </c>
       <c r="I212" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J212" s="8" t="inlineStr">
@@ -8667,7 +8667,7 @@
       </c>
       <c r="I213" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J213" s="12" t="inlineStr">
@@ -8707,7 +8707,7 @@
       </c>
       <c r="I214" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J214" s="8" t="inlineStr">
@@ -8747,7 +8747,7 @@
       </c>
       <c r="I215" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J215" s="12" t="inlineStr">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="I216" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J216" s="8" t="inlineStr">
@@ -8827,7 +8827,7 @@
       </c>
       <c r="I217" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J217" s="12" t="inlineStr">
@@ -8867,7 +8867,7 @@
       </c>
       <c r="I218" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J218" s="8" t="inlineStr">
@@ -8907,7 +8907,7 @@
       </c>
       <c r="I219" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J219" s="12" t="inlineStr">
@@ -8947,7 +8947,7 @@
       </c>
       <c r="I220" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J220" s="8" t="inlineStr">
@@ -8987,7 +8987,7 @@
       </c>
       <c r="I221" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J221" s="12" t="inlineStr">
@@ -9027,7 +9027,7 @@
       </c>
       <c r="I222" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J222" s="8" t="inlineStr">
@@ -9067,7 +9067,7 @@
       </c>
       <c r="I223" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J223" s="12" t="inlineStr">
@@ -9107,7 +9107,7 @@
       </c>
       <c r="I224" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J224" s="8" t="inlineStr">
@@ -9147,7 +9147,7 @@
       </c>
       <c r="I225" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J225" s="12" t="inlineStr">
@@ -9187,7 +9187,7 @@
       </c>
       <c r="I226" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J226" s="8" t="inlineStr">
@@ -9227,7 +9227,7 @@
       </c>
       <c r="I227" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J227" s="12" t="inlineStr">
@@ -9267,7 +9267,7 @@
       </c>
       <c r="I228" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J228" s="8" t="inlineStr">
@@ -9307,7 +9307,7 @@
       </c>
       <c r="I229" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J229" s="12" t="inlineStr">
@@ -9347,7 +9347,7 @@
       </c>
       <c r="I230" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J230" s="8" t="inlineStr">
@@ -9387,7 +9387,7 @@
       </c>
       <c r="I231" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J231" s="12" t="inlineStr">
@@ -9427,7 +9427,7 @@
       </c>
       <c r="I232" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J232" s="8" t="inlineStr">
@@ -9467,7 +9467,7 @@
       </c>
       <c r="I233" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J233" s="12" t="inlineStr">
@@ -9507,7 +9507,7 @@
       </c>
       <c r="I234" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J234" s="8" t="inlineStr">
@@ -9547,7 +9547,7 @@
       </c>
       <c r="I235" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J235" s="12" t="inlineStr">
@@ -9587,7 +9587,7 @@
       </c>
       <c r="I236" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J236" s="8" t="inlineStr">
@@ -9627,7 +9627,7 @@
       </c>
       <c r="I237" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J237" s="12" t="inlineStr">
@@ -9667,7 +9667,7 @@
       </c>
       <c r="I238" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J238" s="8" t="inlineStr">
@@ -9707,7 +9707,7 @@
       </c>
       <c r="I239" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J239" s="12" t="inlineStr">
@@ -9747,7 +9747,7 @@
       </c>
       <c r="I240" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J240" s="8" t="inlineStr">
@@ -9787,7 +9787,7 @@
       </c>
       <c r="I241" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J241" s="12" t="inlineStr">
@@ -9827,7 +9827,7 @@
       </c>
       <c r="I242" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J242" s="8" t="inlineStr">
@@ -9867,7 +9867,7 @@
       </c>
       <c r="I243" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J243" s="12" t="inlineStr">
@@ -9907,7 +9907,7 @@
       </c>
       <c r="I244" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J244" s="8" t="inlineStr">
@@ -9947,7 +9947,7 @@
       </c>
       <c r="I245" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J245" s="12" t="inlineStr">
@@ -9987,7 +9987,7 @@
       </c>
       <c r="I246" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J246" s="8" t="inlineStr">
@@ -10027,7 +10027,7 @@
       </c>
       <c r="I247" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J247" s="12" t="inlineStr">
@@ -10067,7 +10067,7 @@
       </c>
       <c r="I248" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J248" s="8" t="inlineStr">
@@ -10107,7 +10107,7 @@
       </c>
       <c r="I249" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J249" s="12" t="inlineStr">
@@ -10147,7 +10147,7 @@
       </c>
       <c r="I250" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J250" s="8" t="inlineStr">
@@ -10187,7 +10187,7 @@
       </c>
       <c r="I251" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J251" s="12" t="inlineStr">
@@ -10227,7 +10227,7 @@
       </c>
       <c r="I252" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J252" s="8" t="inlineStr">
@@ -10267,7 +10267,7 @@
       </c>
       <c r="I253" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J253" s="12" t="inlineStr">
@@ -10307,7 +10307,7 @@
       </c>
       <c r="I254" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J254" s="8" t="inlineStr">
@@ -10347,7 +10347,7 @@
       </c>
       <c r="I255" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J255" s="12" t="inlineStr">
@@ -10387,7 +10387,7 @@
       </c>
       <c r="I256" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J256" s="8" t="inlineStr">
@@ -10427,7 +10427,7 @@
       </c>
       <c r="I257" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J257" s="12" t="inlineStr">
@@ -10467,7 +10467,7 @@
       </c>
       <c r="I258" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J258" s="8" t="inlineStr">
@@ -10507,7 +10507,7 @@
       </c>
       <c r="I259" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J259" s="12" t="inlineStr">
@@ -10547,7 +10547,7 @@
       </c>
       <c r="I260" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J260" s="8" t="inlineStr">
@@ -10587,7 +10587,7 @@
       </c>
       <c r="I261" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J261" s="12" t="inlineStr">
@@ -10627,7 +10627,7 @@
       </c>
       <c r="I262" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J262" s="8" t="inlineStr">
@@ -10667,7 +10667,7 @@
       </c>
       <c r="I263" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J263" s="12" t="inlineStr">
@@ -10707,7 +10707,7 @@
       </c>
       <c r="I264" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J264" s="8" t="inlineStr">
@@ -10747,7 +10747,7 @@
       </c>
       <c r="I265" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J265" s="12" t="inlineStr">
@@ -10787,7 +10787,7 @@
       </c>
       <c r="I266" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J266" s="8" t="inlineStr">
@@ -10827,7 +10827,7 @@
       </c>
       <c r="I267" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J267" s="12" t="inlineStr">
@@ -10867,7 +10867,7 @@
       </c>
       <c r="I268" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J268" s="8" t="inlineStr">
@@ -10907,7 +10907,7 @@
       </c>
       <c r="I269" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J269" s="12" t="inlineStr">
@@ -10947,7 +10947,7 @@
       </c>
       <c r="I270" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J270" s="8" t="inlineStr">
@@ -10987,7 +10987,7 @@
       </c>
       <c r="I271" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J271" s="12" t="inlineStr">
@@ -11027,7 +11027,7 @@
       </c>
       <c r="I272" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J272" s="8" t="inlineStr">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="I273" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J273" s="12" t="inlineStr">
@@ -11107,7 +11107,7 @@
       </c>
       <c r="I274" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J274" s="8" t="inlineStr">
@@ -11147,7 +11147,7 @@
       </c>
       <c r="I275" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J275" s="12" t="inlineStr">
@@ -11187,7 +11187,7 @@
       </c>
       <c r="I276" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J276" s="8" t="inlineStr">
@@ -11227,7 +11227,7 @@
       </c>
       <c r="I277" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J277" s="12" t="inlineStr">
@@ -11267,7 +11267,7 @@
       </c>
       <c r="I278" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J278" s="8" t="inlineStr">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="I279" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J279" s="12" t="inlineStr">
@@ -11347,7 +11347,7 @@
       </c>
       <c r="I280" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J280" s="8" t="inlineStr">
@@ -11387,7 +11387,7 @@
       </c>
       <c r="I281" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J281" s="12" t="inlineStr">
@@ -11427,7 +11427,7 @@
       </c>
       <c r="I282" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J282" s="8" t="inlineStr">
@@ -11467,7 +11467,7 @@
       </c>
       <c r="I283" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J283" s="12" t="inlineStr">
@@ -11507,7 +11507,7 @@
       </c>
       <c r="I284" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J284" s="8" t="inlineStr">
@@ -11547,7 +11547,7 @@
       </c>
       <c r="I285" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J285" s="12" t="inlineStr">
@@ -11587,7 +11587,7 @@
       </c>
       <c r="I286" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J286" s="8" t="inlineStr">
@@ -11627,7 +11627,7 @@
       </c>
       <c r="I287" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J287" s="12" t="inlineStr">
@@ -11667,7 +11667,7 @@
       </c>
       <c r="I288" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J288" s="8" t="inlineStr">
@@ -11707,7 +11707,7 @@
       </c>
       <c r="I289" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J289" s="12" t="inlineStr">
@@ -11747,7 +11747,7 @@
       </c>
       <c r="I290" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J290" s="8" t="inlineStr">
@@ -11787,7 +11787,7 @@
       </c>
       <c r="I291" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J291" s="12" t="inlineStr">
@@ -11827,7 +11827,7 @@
       </c>
       <c r="I292" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J292" s="8" t="inlineStr">
@@ -11867,7 +11867,7 @@
       </c>
       <c r="I293" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J293" s="12" t="inlineStr">
@@ -11907,7 +11907,7 @@
       </c>
       <c r="I294" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J294" s="8" t="inlineStr">
@@ -11947,7 +11947,7 @@
       </c>
       <c r="I295" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J295" s="12" t="inlineStr">
@@ -11987,7 +11987,7 @@
       </c>
       <c r="I296" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J296" s="8" t="inlineStr">
@@ -12027,7 +12027,7 @@
       </c>
       <c r="I297" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J297" s="12" t="inlineStr">
@@ -12067,7 +12067,7 @@
       </c>
       <c r="I298" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J298" s="8" t="inlineStr">
@@ -12107,7 +12107,7 @@
       </c>
       <c r="I299" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J299" s="12" t="inlineStr">
@@ -12147,7 +12147,7 @@
       </c>
       <c r="I300" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J300" s="8" t="inlineStr">
@@ -12187,7 +12187,7 @@
       </c>
       <c r="I301" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J301" s="12" t="inlineStr">
@@ -12227,7 +12227,7 @@
       </c>
       <c r="I302" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J302" s="8" t="inlineStr">
@@ -12267,7 +12267,7 @@
       </c>
       <c r="I303" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J303" s="12" t="inlineStr">
@@ -12307,7 +12307,7 @@
       </c>
       <c r="I304" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J304" s="8" t="inlineStr">
@@ -12347,7 +12347,7 @@
       </c>
       <c r="I305" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J305" s="12" t="inlineStr">
@@ -12387,7 +12387,7 @@
       </c>
       <c r="I306" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J306" s="8" t="inlineStr">
@@ -12427,7 +12427,7 @@
       </c>
       <c r="I307" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J307" s="12" t="inlineStr">
@@ -12467,7 +12467,7 @@
       </c>
       <c r="I308" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J308" s="8" t="inlineStr">
@@ -12507,7 +12507,7 @@
       </c>
       <c r="I309" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J309" s="12" t="inlineStr">
@@ -12547,7 +12547,7 @@
       </c>
       <c r="I310" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J310" s="8" t="inlineStr">
@@ -12587,7 +12587,7 @@
       </c>
       <c r="I311" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J311" s="12" t="inlineStr">
@@ -12627,7 +12627,7 @@
       </c>
       <c r="I312" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J312" s="8" t="inlineStr">
@@ -12667,7 +12667,7 @@
       </c>
       <c r="I313" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J313" s="12" t="inlineStr">
@@ -12707,7 +12707,7 @@
       </c>
       <c r="I314" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J314" s="8" t="inlineStr">
@@ -12747,7 +12747,7 @@
       </c>
       <c r="I315" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J315" s="12" t="inlineStr">
@@ -12787,7 +12787,7 @@
       </c>
       <c r="I316" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J316" s="8" t="inlineStr">
@@ -12827,7 +12827,7 @@
       </c>
       <c r="I317" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J317" s="12" t="inlineStr">
@@ -12867,7 +12867,7 @@
       </c>
       <c r="I318" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J318" s="8" t="inlineStr">
@@ -12907,7 +12907,7 @@
       </c>
       <c r="I319" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J319" s="12" t="inlineStr">
@@ -12947,7 +12947,7 @@
       </c>
       <c r="I320" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J320" s="8" t="inlineStr">
@@ -12987,7 +12987,7 @@
       </c>
       <c r="I321" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J321" s="12" t="inlineStr">
@@ -13027,7 +13027,7 @@
       </c>
       <c r="I322" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J322" s="8" t="inlineStr">
@@ -13067,7 +13067,7 @@
       </c>
       <c r="I323" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J323" s="12" t="inlineStr">
@@ -13107,7 +13107,7 @@
       </c>
       <c r="I324" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J324" s="8" t="inlineStr">
@@ -13147,7 +13147,7 @@
       </c>
       <c r="I325" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J325" s="12" t="inlineStr">
@@ -13187,7 +13187,7 @@
       </c>
       <c r="I326" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J326" s="8" t="inlineStr">
@@ -13227,7 +13227,7 @@
       </c>
       <c r="I327" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J327" s="12" t="inlineStr">
@@ -13267,7 +13267,7 @@
       </c>
       <c r="I328" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J328" s="8" t="inlineStr">
@@ -13307,7 +13307,7 @@
       </c>
       <c r="I329" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J329" s="12" t="inlineStr">
@@ -13347,7 +13347,7 @@
       </c>
       <c r="I330" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J330" s="8" t="inlineStr">
@@ -13387,7 +13387,7 @@
       </c>
       <c r="I331" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J331" s="12" t="inlineStr">
@@ -13427,7 +13427,7 @@
       </c>
       <c r="I332" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J332" s="8" t="inlineStr">
@@ -13467,7 +13467,7 @@
       </c>
       <c r="I333" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J333" s="12" t="inlineStr">
@@ -13507,7 +13507,7 @@
       </c>
       <c r="I334" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J334" s="8" t="inlineStr">
@@ -13547,7 +13547,7 @@
       </c>
       <c r="I335" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J335" s="12" t="inlineStr">
@@ -13587,7 +13587,7 @@
       </c>
       <c r="I336" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J336" s="8" t="inlineStr">
@@ -13627,7 +13627,7 @@
       </c>
       <c r="I337" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J337" s="12" t="inlineStr">
@@ -13667,7 +13667,7 @@
       </c>
       <c r="I338" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J338" s="8" t="inlineStr">
@@ -13707,7 +13707,7 @@
       </c>
       <c r="I339" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J339" s="12" t="inlineStr">
@@ -13747,7 +13747,7 @@
       </c>
       <c r="I340" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J340" s="8" t="inlineStr">
@@ -13787,7 +13787,7 @@
       </c>
       <c r="I341" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J341" s="12" t="inlineStr">
@@ -13827,7 +13827,7 @@
       </c>
       <c r="I342" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J342" s="8" t="inlineStr">
@@ -13867,7 +13867,7 @@
       </c>
       <c r="I343" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J343" s="12" t="inlineStr">
@@ -13907,7 +13907,7 @@
       </c>
       <c r="I344" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J344" s="8" t="inlineStr">
@@ -13947,7 +13947,7 @@
       </c>
       <c r="I345" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J345" s="12" t="inlineStr">
@@ -13987,7 +13987,7 @@
       </c>
       <c r="I346" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J346" s="8" t="inlineStr">
@@ -14027,7 +14027,7 @@
       </c>
       <c r="I347" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J347" s="12" t="inlineStr">
@@ -14067,7 +14067,7 @@
       </c>
       <c r="I348" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J348" s="8" t="inlineStr">
@@ -14107,7 +14107,7 @@
       </c>
       <c r="I349" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J349" s="12" t="inlineStr">
@@ -14147,7 +14147,7 @@
       </c>
       <c r="I350" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J350" s="8" t="inlineStr">
@@ -14187,7 +14187,7 @@
       </c>
       <c r="I351" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J351" s="12" t="inlineStr">
@@ -14227,7 +14227,7 @@
       </c>
       <c r="I352" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J352" s="8" t="inlineStr">
@@ -14267,7 +14267,7 @@
       </c>
       <c r="I353" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J353" s="12" t="inlineStr">
@@ -14307,7 +14307,7 @@
       </c>
       <c r="I354" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J354" s="8" t="inlineStr">
@@ -14347,7 +14347,7 @@
       </c>
       <c r="I355" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J355" s="12" t="inlineStr">
@@ -14387,7 +14387,7 @@
       </c>
       <c r="I356" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J356" s="8" t="inlineStr">
@@ -14427,7 +14427,7 @@
       </c>
       <c r="I357" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J357" s="12" t="inlineStr">
@@ -14467,7 +14467,7 @@
       </c>
       <c r="I358" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J358" s="8" t="inlineStr">
@@ -14507,7 +14507,7 @@
       </c>
       <c r="I359" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J359" s="12" t="inlineStr">
@@ -14547,7 +14547,7 @@
       </c>
       <c r="I360" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J360" s="8" t="inlineStr">
@@ -14587,7 +14587,7 @@
       </c>
       <c r="I361" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J361" s="12" t="inlineStr">
@@ -14627,7 +14627,7 @@
       </c>
       <c r="I362" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J362" s="8" t="inlineStr">
@@ -14667,7 +14667,7 @@
       </c>
       <c r="I363" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J363" s="12" t="inlineStr">
@@ -14707,7 +14707,7 @@
       </c>
       <c r="I364" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J364" s="8" t="inlineStr">
@@ -14747,7 +14747,7 @@
       </c>
       <c r="I365" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J365" s="12" t="inlineStr">
@@ -14787,7 +14787,7 @@
       </c>
       <c r="I366" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J366" s="8" t="inlineStr">
@@ -14827,7 +14827,7 @@
       </c>
       <c r="I367" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J367" s="12" t="inlineStr">
@@ -14867,7 +14867,7 @@
       </c>
       <c r="I368" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J368" s="8" t="inlineStr">
@@ -14907,7 +14907,7 @@
       </c>
       <c r="I369" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J369" s="12" t="inlineStr">
@@ -14947,7 +14947,7 @@
       </c>
       <c r="I370" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J370" s="8" t="inlineStr">
@@ -14987,7 +14987,7 @@
       </c>
       <c r="I371" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J371" s="12" t="inlineStr">
@@ -15027,7 +15027,7 @@
       </c>
       <c r="I372" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J372" s="8" t="inlineStr">
@@ -15067,7 +15067,7 @@
       </c>
       <c r="I373" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J373" s="12" t="inlineStr">
@@ -15107,7 +15107,7 @@
       </c>
       <c r="I374" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J374" s="8" t="inlineStr">
@@ -15147,7 +15147,7 @@
       </c>
       <c r="I375" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J375" s="12" t="inlineStr">
@@ -15187,7 +15187,7 @@
       </c>
       <c r="I376" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J376" s="8" t="inlineStr">
@@ -15227,7 +15227,7 @@
       </c>
       <c r="I377" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J377" s="12" t="inlineStr">
@@ -15267,7 +15267,7 @@
       </c>
       <c r="I378" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J378" s="8" t="inlineStr">
@@ -15307,7 +15307,7 @@
       </c>
       <c r="I379" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J379" s="12" t="inlineStr">
@@ -15347,7 +15347,7 @@
       </c>
       <c r="I380" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J380" s="8" t="inlineStr">
@@ -15387,7 +15387,7 @@
       </c>
       <c r="I381" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J381" s="12" t="inlineStr">
@@ -15427,7 +15427,7 @@
       </c>
       <c r="I382" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J382" s="8" t="inlineStr">
@@ -15467,7 +15467,7 @@
       </c>
       <c r="I383" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J383" s="12" t="inlineStr">
@@ -15507,7 +15507,7 @@
       </c>
       <c r="I384" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J384" s="8" t="inlineStr">
@@ -15547,7 +15547,7 @@
       </c>
       <c r="I385" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J385" s="12" t="inlineStr">
@@ -15587,7 +15587,7 @@
       </c>
       <c r="I386" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J386" s="8" t="inlineStr">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="I387" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J387" s="12" t="inlineStr">
@@ -15667,7 +15667,7 @@
       </c>
       <c r="I388" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J388" s="8" t="inlineStr">
@@ -15707,7 +15707,7 @@
       </c>
       <c r="I389" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J389" s="12" t="inlineStr">
@@ -15747,7 +15747,7 @@
       </c>
       <c r="I390" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J390" s="8" t="inlineStr">
@@ -15787,7 +15787,7 @@
       </c>
       <c r="I391" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J391" s="12" t="inlineStr">
@@ -15827,7 +15827,7 @@
       </c>
       <c r="I392" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J392" s="8" t="inlineStr">
@@ -15867,7 +15867,7 @@
       </c>
       <c r="I393" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J393" s="12" t="inlineStr">
@@ -15907,7 +15907,7 @@
       </c>
       <c r="I394" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J394" s="8" t="inlineStr">
@@ -15947,7 +15947,7 @@
       </c>
       <c r="I395" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J395" s="12" t="inlineStr">
@@ -15987,7 +15987,7 @@
       </c>
       <c r="I396" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J396" s="8" t="inlineStr">
@@ -16027,7 +16027,7 @@
       </c>
       <c r="I397" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J397" s="12" t="inlineStr">
@@ -16067,7 +16067,7 @@
       </c>
       <c r="I398" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J398" s="8" t="inlineStr">
@@ -16107,7 +16107,7 @@
       </c>
       <c r="I399" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J399" s="12" t="inlineStr">
@@ -16147,7 +16147,7 @@
       </c>
       <c r="I400" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J400" s="8" t="inlineStr">
@@ -16187,7 +16187,7 @@
       </c>
       <c r="I401" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J401" s="12" t="inlineStr">
@@ -16227,7 +16227,7 @@
       </c>
       <c r="I402" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J402" s="8" t="inlineStr">
@@ -16267,7 +16267,7 @@
       </c>
       <c r="I403" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J403" s="12" t="inlineStr">
@@ -16307,7 +16307,7 @@
       </c>
       <c r="I404" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J404" s="8" t="inlineStr">
@@ -16347,7 +16347,7 @@
       </c>
       <c r="I405" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J405" s="12" t="inlineStr">
@@ -16387,7 +16387,7 @@
       </c>
       <c r="I406" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J406" s="8" t="inlineStr">
@@ -16427,7 +16427,7 @@
       </c>
       <c r="I407" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J407" s="12" t="inlineStr">
@@ -16467,7 +16467,7 @@
       </c>
       <c r="I408" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J408" s="8" t="inlineStr">
@@ -16507,7 +16507,7 @@
       </c>
       <c r="I409" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J409" s="12" t="inlineStr">
@@ -16547,7 +16547,7 @@
       </c>
       <c r="I410" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J410" s="8" t="inlineStr">
@@ -16587,7 +16587,7 @@
       </c>
       <c r="I411" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J411" s="12" t="inlineStr">
@@ -16627,7 +16627,7 @@
       </c>
       <c r="I412" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J412" s="8" t="inlineStr">
@@ -16667,7 +16667,7 @@
       </c>
       <c r="I413" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J413" s="12" t="inlineStr">
@@ -16707,7 +16707,7 @@
       </c>
       <c r="I414" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J414" s="8" t="inlineStr">
@@ -16747,7 +16747,7 @@
       </c>
       <c r="I415" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J415" s="12" t="inlineStr">
@@ -16787,7 +16787,7 @@
       </c>
       <c r="I416" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J416" s="8" t="inlineStr">
@@ -16827,7 +16827,7 @@
       </c>
       <c r="I417" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J417" s="12" t="inlineStr">
@@ -16867,7 +16867,7 @@
       </c>
       <c r="I418" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J418" s="8" t="inlineStr">
@@ -16907,7 +16907,7 @@
       </c>
       <c r="I419" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J419" s="12" t="inlineStr">
@@ -16947,7 +16947,7 @@
       </c>
       <c r="I420" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J420" s="8" t="inlineStr">
@@ -16987,7 +16987,7 @@
       </c>
       <c r="I421" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J421" s="12" t="inlineStr">
@@ -17027,7 +17027,7 @@
       </c>
       <c r="I422" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J422" s="8" t="inlineStr">
@@ -17067,7 +17067,7 @@
       </c>
       <c r="I423" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J423" s="12" t="inlineStr">
@@ -17107,7 +17107,7 @@
       </c>
       <c r="I424" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J424" s="8" t="inlineStr">
@@ -17147,7 +17147,7 @@
       </c>
       <c r="I425" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J425" s="12" t="inlineStr">
@@ -17187,7 +17187,7 @@
       </c>
       <c r="I426" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J426" s="8" t="inlineStr">
@@ -17227,7 +17227,7 @@
       </c>
       <c r="I427" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J427" s="12" t="inlineStr">
@@ -17267,7 +17267,7 @@
       </c>
       <c r="I428" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J428" s="8" t="inlineStr">
@@ -17307,7 +17307,7 @@
       </c>
       <c r="I429" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J429" s="12" t="inlineStr">
@@ -17347,7 +17347,7 @@
       </c>
       <c r="I430" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J430" s="8" t="inlineStr">
@@ -17387,7 +17387,7 @@
       </c>
       <c r="I431" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J431" s="12" t="inlineStr">
@@ -17427,7 +17427,7 @@
       </c>
       <c r="I432" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J432" s="8" t="inlineStr">
@@ -17467,7 +17467,7 @@
       </c>
       <c r="I433" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J433" s="12" t="inlineStr">
@@ -17507,7 +17507,7 @@
       </c>
       <c r="I434" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J434" s="8" t="inlineStr">
@@ -17547,7 +17547,7 @@
       </c>
       <c r="I435" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J435" s="12" t="inlineStr">
@@ -17587,7 +17587,7 @@
       </c>
       <c r="I436" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J436" s="8" t="inlineStr">
@@ -17627,7 +17627,7 @@
       </c>
       <c r="I437" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J437" s="12" t="inlineStr">
@@ -17667,7 +17667,7 @@
       </c>
       <c r="I438" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J438" s="8" t="inlineStr">
@@ -17707,7 +17707,7 @@
       </c>
       <c r="I439" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J439" s="12" t="inlineStr">
@@ -17747,7 +17747,7 @@
       </c>
       <c r="I440" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J440" s="8" t="inlineStr">
@@ -17787,7 +17787,7 @@
       </c>
       <c r="I441" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J441" s="12" t="inlineStr">
@@ -17827,7 +17827,7 @@
       </c>
       <c r="I442" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J442" s="8" t="inlineStr">
@@ -17867,7 +17867,7 @@
       </c>
       <c r="I443" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J443" s="12" t="inlineStr">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="I444" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J444" s="8" t="inlineStr">
@@ -17947,7 +17947,7 @@
       </c>
       <c r="I445" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J445" s="12" t="inlineStr">
@@ -17987,7 +17987,7 @@
       </c>
       <c r="I446" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J446" s="8" t="inlineStr">
@@ -18027,7 +18027,7 @@
       </c>
       <c r="I447" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J447" s="12" t="inlineStr">
@@ -18067,7 +18067,7 @@
       </c>
       <c r="I448" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J448" s="8" t="inlineStr">
@@ -18107,7 +18107,7 @@
       </c>
       <c r="I449" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J449" s="12" t="inlineStr">
@@ -18147,7 +18147,7 @@
       </c>
       <c r="I450" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J450" s="8" t="inlineStr">
@@ -18187,7 +18187,7 @@
       </c>
       <c r="I451" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J451" s="12" t="inlineStr">
@@ -18227,7 +18227,7 @@
       </c>
       <c r="I452" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J452" s="8" t="inlineStr">
@@ -18267,7 +18267,7 @@
       </c>
       <c r="I453" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J453" s="12" t="inlineStr">
@@ -18307,7 +18307,7 @@
       </c>
       <c r="I454" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J454" s="8" t="inlineStr">
@@ -18347,7 +18347,7 @@
       </c>
       <c r="I455" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J455" s="12" t="inlineStr">
@@ -18387,7 +18387,7 @@
       </c>
       <c r="I456" s="8" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J456" s="8" t="inlineStr">
@@ -18427,7 +18427,7 @@
       </c>
       <c r="I457" s="12" t="inlineStr">
         <is>
-          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/{CCBFCEE4-FB9B-F179-93C3-F376FBE5491F}.pdf</t>
+          <t>https://www.banxico.org.mx/publicaciones-y-prensa/estado-de-cuenta-semanal/estado-cuenta-semanal-reserva.html</t>
         </is>
       </c>
       <c r="J457" s="12" t="inlineStr">

</xml_diff>